<commit_message>
fix: align final project records with supplied template
</commit_message>
<xml_diff>
--- a/Hours_on_Project.xlsx
+++ b/Hours_on_Project.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hours" sheetId="1" r:id="R62a9145282464a87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hours" sheetId="1" r:id="Rd64af1ec7dd44430"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -903,7 +903,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="115" t="str">
-        <x:v>Nexus Five - Team 5 | 21 May-2 August 2026</x:v>
+        <x:v>Nexus Five | 21 May-2 August 2026</x:v>
       </x:c>
       <x:c r="B2" s="115"/>
       <x:c r="C2" s="115"/>
@@ -914,7 +914,7 @@
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
       <x:c r="A3" s="89" t="str">
-        <x:v>Final allocation uses half-hour increments and reflects role-based variation.</x:v>
+        <x:v>Weekly hours include meetings, documentation, design, implementation, review, and final submission work.</x:v>
       </x:c>
       <x:c r="B3" s="89"/>
       <x:c r="C3" s="89"/>
@@ -923,14 +923,14 @@
       </x:c>
       <x:c r="E3" s="117" t="n">
         <x:f>F31</x:f>
-        <x:v>150</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="F3" s="118" t="str">
         <x:v>Actual total</x:v>
       </x:c>
       <x:c r="G3" s="119" t="n">
         <x:f>F32</x:f>
-        <x:v>150</x:v>
+        <x:v>591</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -974,19 +974,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C6" s="124" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D6" s="124" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E6" s="124" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F6" s="124" t="n">
-        <x:v>1.5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G6" s="125" t="n">
-        <x:v>1.5</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
@@ -995,19 +995,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C7" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E7" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F7" s="128" t="n">
-        <x:v>1.5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G7" s="129" t="n">
-        <x:v>1.5</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
@@ -1019,19 +1019,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C8" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D8" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E8" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F8" s="124" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G8" s="125" t="n">
-        <x:v>2.5</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
@@ -1040,19 +1040,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C9" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D9" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E9" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F9" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G9" s="129" t="n">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
@@ -1064,19 +1064,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C10" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D10" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E10" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F10" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G10" s="125" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
@@ -1085,19 +1085,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C11" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D11" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E11" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F11" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G11" s="129" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
@@ -1109,19 +1109,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C12" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D12" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E12" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F12" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G12" s="125" t="n">
-        <x:v>3</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
@@ -1130,19 +1130,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C13" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D13" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E13" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F13" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G13" s="129" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
@@ -1154,19 +1154,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C14" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D14" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E14" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F14" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G14" s="125" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
@@ -1175,19 +1175,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C15" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D15" s="128" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E15" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F15" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G15" s="129" t="n">
-        <x:v>2.5</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
@@ -1199,19 +1199,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C16" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D16" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E16" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F16" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G16" s="125" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
@@ -1220,19 +1220,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C17" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D17" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E17" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F17" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G17" s="129" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
@@ -1244,19 +1244,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C18" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D18" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E18" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F18" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G18" s="125" t="n">
-        <x:v>3.5</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
@@ -1265,19 +1265,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C19" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D19" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E19" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F19" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G19" s="129" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
@@ -1289,19 +1289,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C20" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D20" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E20" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F20" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G20" s="125" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
@@ -1310,19 +1310,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C21" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D21" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E21" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F21" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G21" s="129" t="n">
-        <x:v>3</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
@@ -1334,19 +1334,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C22" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D22" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E22" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F22" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G22" s="125" t="n">
-        <x:v>3</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
@@ -1355,19 +1355,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C23" s="128" t="n">
-        <x:v>4</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D23" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E23" s="128" t="n">
-        <x:v>4</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F23" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G23" s="129" t="n">
-        <x:v>3</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
@@ -1379,19 +1379,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C24" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D24" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E24" s="124" t="n">
-        <x:v>3.5</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="F24" s="124" t="n">
-        <x:v>3</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G24" s="125" t="n">
-        <x:v>4</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
@@ -1400,19 +1400,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C25" s="128" t="n">
-        <x:v>4</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D25" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E25" s="128" t="n">
-        <x:v>3.5</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F25" s="128" t="n">
-        <x:v>3</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="G25" s="129" t="n">
-        <x:v>3.5</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
@@ -1424,19 +1424,19 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="C26" s="124" t="n">
-        <x:v>1.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D26" s="124" t="n">
-        <x:v>1.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E26" s="124" t="n">
-        <x:v>1.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F26" s="124" t="n">
-        <x:v>2.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G26" s="125" t="n">
-        <x:v>1.5</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
@@ -1445,19 +1445,19 @@
         <x:v>Actual</x:v>
       </x:c>
       <x:c r="C27" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D27" s="128" t="n">
-        <x:v>1.5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E27" s="128" t="n">
-        <x:v>1.5</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="F27" s="128" t="n">
-        <x:v>2</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="G27" s="129" t="n">
-        <x:v>1.5</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -1469,23 +1469,23 @@
       </x:c>
       <x:c r="C28" s="131" t="n">
         <x:f>SUM(C6,C8,C10,C12,C14,C16,C18,C20,C22,C24,C26)</x:f>
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D28" s="131" t="n">
         <x:f>SUM(D6,D8,D10,D12,D14,D16,D18,D20,D22,D24,D26)</x:f>
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E28" s="131" t="n">
         <x:f>SUM(E6,E8,E10,E12,E14,E16,E18,E20,E22,E24,E26)</x:f>
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="F28" s="131" t="n">
         <x:f>SUM(F6,F8,F10,F12,F14,F16,F18,F20,F22,F24,F26)</x:f>
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="G28" s="131" t="n">
         <x:f>SUM(G6,G8,G10,G12,G14,G16,G18,G20,G22,G24,G26)</x:f>
-        <x:v>30</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
@@ -1495,23 +1495,23 @@
       </x:c>
       <x:c r="C29" s="131" t="n">
         <x:f>SUM(C7,C9,C11,C13,C15,C17,C19,C21,C23,C25,C27)</x:f>
-        <x:v>32</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="D29" s="131" t="n">
         <x:f>SUM(D7,D9,D11,D13,D15,D17,D19,D21,D23,D25,D27)</x:f>
-        <x:v>30</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E29" s="131" t="n">
         <x:f>SUM(E7,E9,E11,E13,E15,E17,E19,E21,E23,E25,E27)</x:f>
-        <x:v>31</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F29" s="131" t="n">
         <x:f>SUM(F7,F9,F11,F13,F15,F17,F19,F21,F23,F25,F27)</x:f>
-        <x:v>29</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="G29" s="131" t="n">
         <x:f>SUM(G7,G9,G11,G13,G15,G17,G19,G21,G23,G25,G27)</x:f>
-        <x:v>28</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1533,7 +1533,7 @@
       <x:c r="E31" s="133"/>
       <x:c r="F31" s="134" t="n">
         <x:f>SUM(C28:G28)</x:f>
-        <x:v>150</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="G31" s="135" t="str">
         <x:v>hours</x:v>
@@ -1549,7 +1549,7 @@
       <x:c r="E32" s="137"/>
       <x:c r="F32" s="138" t="n">
         <x:f>SUM(C29:G29)</x:f>
-        <x:v>150</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="G32" s="139" t="str">
         <x:v>hours</x:v>

</xml_diff>